<commit_message>
Release v1.3: XS migration + KB reconciliation + web-format standards
AS/ES->XS series-ID migration; line-by-line KB reconciliation (fabricated
citations corrected, culled series removed); per-subseries units; CSV+parquet
downloads; Anu Explainers; internal handoff/build artifacts removed from the
public bundle.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/extenbooks/S201.xlsx
+++ b/extenbooks/S201.xlsx
@@ -451,7 +451,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,7 +462,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>S&amp;T 1994, units=billions_usd</t>
+          <t>S&amp;T 1994, units=ratio</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
         <v>1954</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.858278986759664</v>
+        <v>0.8584326166498955</v>
       </c>
     </row>
     <row r="10">
@@ -825,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -900,7 +900,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>billions_usd</t>
+          <t>ratio</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>cross_sectional</t>
+          <t>time_series</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t>- **Chapter**: 2 (Theoretical framework for the production/nonproduction distinction; book Figure 1.1, Table 2.1)</t>
+          <t>- **Chapter**: 2 (theoretical framework for the production/nonproduction distinction; book Figure 1.1). **Note**: there is NO book Table 2.1 — the book's List of Tables (folios xi–xii) begins at Table 3.1; Chapter 2 is purely theoretical and contains no tables. The earlier "Table 2.1 (Alternative GFP Measures)" citation was a hallucination (removed 2026-06-11, triage patch S201). The in-book analog of S201 is Figure 5.4 ("Ratios of real product measures", folio 106) and the Table 5.4 row GFP*/GNP (folio 100); the name "Alternative GFP Measures" derives from Figure 1.1 ("Alternate measures of GFP", folio 16).</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>- **Status**: `book_period_validated` (extension block null pending Wave 3 implementation of post-1989 NIPA mapping)</t>
+          <t>- **Status**: book_period_validated</t>
         </is>
       </c>
     </row>
@@ -1078,87 +1078,87 @@
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>- **Units**: ratio (GFP/GDP and FP/NDP) and billions of current dollars (Marxian GFP* level)</t>
+          <t>- **Status note**: (extension block null pending Wave 3 implementation of post-1989 NIPA mapping)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>- **Units**: ratio (GFP/GDP and FP/NDP) and billions of current dollars (Marxian GFP* level)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>## Methodology</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>## Methodology</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>S201 operationalizes the Shaikh-Tonak (S&amp;T) Marxian Gross Final Product (GFP*) by comparing it against orthodox BEA national-accounting aggregates. Two ratio series are constructed annually 1948-1989: `GFP_GDP_ratio = S503 / GDP` and `FP_NDP_ratio = (S503 - CFC_productive) / NDP`. The numerator S503 is the project's Wave-1 Marxian GFP* series, built upstream from the same BEA Tables 1.7.5 / 1.14 used here for the denominator. The headline finding is that the ratio falls over the postwar period from approximately 0.903 (1948) to 0.773 (1989), indicating the unproductive share of GDP — finance, business services, government administration, retail margins — is growing faster than the productive sectors.</t>
-        </is>
-      </c>
+      <c r="B31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
-      <c r="B32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>S201 operationalizes the Shaikh-Tonak (S&amp;T) Marxian Gross Final Product (GFP*) by comparing it against orthodox BEA national-accounting aggregates. Two ratio series are constructed annually 1948-1989: `GFP_GDP_ratio = S503 / GDP` and `FP_NDP_ratio = (S503 - CFC_productive) / NDP`. The numerator S503 is the project's Wave-1 Marxian GFP* series, built upstream from the same BEA Tables 1.7.5 / 1.14 used here for the denominator. The headline finding is that the ratio falls over the postwar period from approximately 0.903 (1948) to 0.773 (1989), indicating the unproductive share of GDP — finance, business services, government administration, retail margins — is growing faster than the productive sectors.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>The theoretical foundation is the S&amp;T production boundary: production activities use existing wealth to create new wealth (use-values), while distribution (trading, wholesale/retail, advertising), social maintenance (military, police, administration), and personal consumption are forms of social consumption that use up wealth without creating new wealth. Under capitalism the productive-labor condition is further restricted to wage labor exchanged against capital. The book is explicit that the distinction is not between goods and services: most service activities (transportation, lodging, repairs, productive entertainment) are classified as production, while many activities conventionally counted as "output" (wholesale/retail margins, financial intermediation, legal services, civil service) are excluded. The book's Figure 1.1 (p.16) compares seven alternative GFP estimates against BEA GNP for the mid-1960s benchmark: NT, Z, JF, K, R, E, and ST. All seven exceed official GNP; S&amp;T's preferred pure-market estimate is approximately 121% of GNP, rising to ~180% when Eisner's housework imputation is added for comparability. The verbatim foundation is **"The location of the dividing line between production and nonproduction activities … changes the very measures of net product, surplus product, consumption, investment, and productivity. The observed trends of these and many other critical variables are also quite different from those in conventional accounts."** (ST 1994, Ch1 §1.4, p.19) and **"What distinguishes the classical/Marxian tradition from the neoclassical/Keynesian one is the location of the dividing line. The former places distribution and social maintenance activities in the sphere of nonproduction activities, whereas the latter places them in production."** (ST 1994, Ch2 §2.1.3, p.25).</t>
-        </is>
-      </c>
+      <c r="B33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>The theoretical foundation is the S&amp;T production boundary: production activities use existing wealth to create new wealth (use-values), while distribution (trading, wholesale/retail, advertising), social maintenance (military, police, administration), and personal consumption are forms of social consumption that use up wealth without creating new wealth. Under capitalism the productive-labor condition is further restricted to wage labor exchanged against capital. The book is explicit that the distinction is not between goods and services: most service activities (transportation, lodging, repairs, productive entertainment) are classified as production, while many activities conventionally counted as "output" (wholesale/retail margins, financial intermediation, legal services, civil service) are excluded. The book's Figure 1.1 (p.16) compares seven alternative GFP estimates against BEA GNP for the mid-1960s benchmark: NT, Z, JF, K, R, E, and ST. All seven exceed official GNP; S&amp;T's preferred pure-market estimate is approximately 121% of GNP, rising to ~180% when Eisner's housework imputation is added for comparability. The verbatim foundation is **"The location of the dividing line between production and nonproduction activities … changes the very measures of net product, surplus product, consumption, investment, and productivity. The observed trends of these and many other critical variables are also quite different from those in conventional accounts."** (ST 1994, Ch1 §1.4, p.19) and **"What distinguishes the classical/Marxian tradition from the neoclassical/Keynesian one is the location of the dividing line. The former places distribution and social maintenance activities in the sphere of nonproduction activities, whereas the latter places them in production."** (ST 1994, Ch2 §2.1.3, p.25).</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>The construction departs from S&amp;T's Figure 1.1 in scope only: rather than the seven-author cross-section at one benchmark year, S201 produces an annual 1948-1989 panel of the ST vs orthodox ratio. The book table that S201 most directly mirrors is Table 2.1 ("Alternative GFP Measures"), still pending full digitization at `data/source/book_tables/ch02/Table2_1_AlternativeGFP.csv`. The pipeline reads cached BEA NIPA Table 1.7.5 (lines 1 GDP, 4 GNP, 5 CFC, 14 NDP, 16 NI) and the upstream S503 final CSV, then computes the two ratios per year. Validation against `expected_range=[0.6, 1.0]` passes for the full book period (observed range 0.773-0.903).</t>
-        </is>
-      </c>
+      <c r="B35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>The construction departs from S&amp;T's Figure 1.1 in scope only: rather than the seven-author cross-section at one benchmark year, S201 produces an annual 1948-1989 panel of the ST vs orthodox ratio. S201 is a DERIVED ratio (S503/GDP), not a digitized book table; the book has no Table 2.1. The in-book analog is Figure 5.4 ("Ratios of real product measures", folio 106) and the Table 5.4 row GFP*/GNP (folio 100). The pipeline reads cached BEA NIPA Table 1.7.5 (lines 1 GDP, 4 GNP, 5 CFC, 14 NDP, 16 NI) and the upstream S503 final CSV, then computes the two ratios per year. Validation against `expected_range=[0.6, 1.0]` passes for the full book period (observed range 0.773-0.903).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>## Sources</t>
-        </is>
-      </c>
+      <c r="B37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>## Sources</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>- KB chunks: `Inputs/Shaikh Tonak/Knowledge_Base/HDARP_Extractions/1994_Measuring_Wealth/chunk_03/full_transcription.md` (Ch1 §1.1, pp.2-5 — classical vs neoclassical boundary); `chunk_04/full_transcription.md` (Ch1 §1.4, pp.15-19 — Figure 1.1 comparison of seven estimates); `chunk_05/full_transcription.md` (Ch2 §2.1, pp.21-30 — production boundary); `chunk_26/full_transcription.md` (Appendix A pp.232-241 — BEA benchmark IO database)</t>
-        </is>
-      </c>
+      <c r="B39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>- Book tables: ST 1994 Table 2.1 (Alternative GFP Measures, annual 1948-1989); Table 5.4 (underlying ST market-production estimate); Figure 1.1 (seven-author comparison, p.16)</t>
+          <t>- KB chunks: `Inputs/Shaikh Tonak/Knowledge_Base/HDARP_Extractions/1994_Measuring_Wealth/chunk_03/full_transcription.md` (Ch1 §1.1, pp.2-5 — classical vs neoclassical boundary); `chunk_04/full_transcription.md` (Ch1 §1.4, pp.15-19 — Figure 1.1 comparison of seven estimates); `chunk_05/full_transcription.md` (Ch2 §2.1, pp.21-30 — production boundary); `chunk_26/full_transcription.md` (Appendix A pp.232-241 — BEA benchmark IO database)</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1166,7 @@
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
-          <t>- External sources: Eisner (1988, JEL, table S.5, p.1673 — comparative GFP estimates); Eisner (1985, p.36 — housework imputation $267.9B in 1966)</t>
+          <t>- Book tables/figures: ST 1994 Table 5.4 (Primary Marxian and NIPA measures, 1948-89, folio 100, row GFP*/GNP); Figure 5.4 (Ratios of real product measures, folio 106); Figure 1.1 (seven-author "Alternate measures of GFP" comparison, folio 16). (There is NO book Table 2.1; the prior citation was a hallucination, removed 2026-06-11.)</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
-          <t>- APIs: BEA NIPA Table 1.7.5 (lines 1, 4, 5, 14, 16); Table 1.14 — cached locally for 1929-2024</t>
+          <t>- External sources: Eisner (1988, JEL, table S.5, p.1673 — comparative GFP estimates); Eisner (1985, p.36 — housework imputation $267.9B in 1966)</t>
         </is>
       </c>
     </row>
@@ -1182,39 +1182,39 @@
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>- Upstream series: S503 final CSV (Marxian GFP*)</t>
+          <t>- APIs: BEA NIPA Table 1.7.5 (lines 1, 4, 5, 14, 16); Table 1.14 — cached locally for 1929-2024</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>- Upstream series: S503 final CSV (Marxian GFP*)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>## Reference values</t>
-        </is>
-      </c>
+      <c r="B45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>## Reference values</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>- 1948: `GFP_GDP_ratio = 0.903`</t>
-        </is>
-      </c>
+      <c r="B47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
-          <t>- 1989: `GFP_GDP_ratio = 0.773`</t>
+          <t>- 1948: `GFP_GDP_ratio = 0.903`</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
-          <t>- 1966 (Figure 1.1 cross-section): ST pure-market GFP/GNP ≈ 1.21; ST + Eisner housework GFP/GNP ≈ 1.80</t>
+          <t>- 1989: `GFP_GDP_ratio = 0.773`</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
-          <t>- Expected range over book period: `[0.6, 1.0]` (validator-enforced)</t>
+          <t>- 1966 (Figure 1.1 cross-section): ST pure-market GFP/GNP ≈ 1.21; ST + Eisner housework GFP/GNP ≈ 1.80</t>
         </is>
       </c>
     </row>
@@ -1238,39 +1238,39 @@
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
-          <t>- Direction: monotonic decline 1948→1989 (unproductive share rising)</t>
+          <t>- Expected range over book period: `[0.6, 1.0]` (validator-enforced)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>- Direction: monotonic decline 1948→1989 (unproductive share rising)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>## Known issues</t>
-        </is>
-      </c>
+      <c r="B53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>## Known issues</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>- Series was originally `wave3_planned`; per the 2026-05-19 honesty pass it is now `book_period_validated` with `extension: null` (no post-1989 build yet; would require either continued NIPA mapping or a NAICS-era productive/unproductive concordance)</t>
-        </is>
-      </c>
+      <c r="B55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
-          <t>- Source CSV `data/source/book_tables/ch02/Table2_1_AlternativeGFP.csv` for the printed book Table 2.1 is not yet digitized; current implementation derives the ratios live from BEA NIPA + S503 rather than from the printed table</t>
+          <t>- Series was originally `wave3_planned`; per the 2026-05-19 honesty pass it is now `book_period_validated` with `extension: null` (no post-1989 build yet; would require either continued NIPA mapping or a NAICS-era productive/unproductive concordance)</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr">
         <is>
-          <t>- Figure 1.1 comparison uses different benchmark years across authors (1965 for NT/Z; 1966 for JF/K/E/ST; 1969 for R), limiting strict cross-author comparability for the benchmark snapshot</t>
+          <t>- S201 is computed live from BEA NIPA + S503 (a derived ratio), not loaded from any digitized book table. There is no printed book Table 2.1 and no `ch02/Table2_1_AlternativeGFP.csv` — the earlier "pending digitization" note referred to a hallucinated table and is void.</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
-          <t>- ST's preferred pure-market estimate (~121% of GNP) differs from the housework-supplemented estimate (~180%) shown in Figure 1.1 for comparability purposes; the housework supplement is not part of S&amp;T's recommended measure</t>
+          <t>- Figure 1.1 comparison uses different benchmark years across authors (1965 for NT/Z; 1966 for JF/K/E/ST; 1969 for R), limiting strict cross-author comparability for the benchmark snapshot</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
-          <t>- Reference values dict in `series_registry.json` is currently empty (this DPR is the authoritative benchmark record pending registry patch)</t>
+          <t>- ST's preferred pure-market estimate (~121% of GNP) differs from the housework-supplemented estimate (~180%) shown in Figure 1.1 for comparability purposes; the housework supplement is not part of S&amp;T's recommended measure</t>
         </is>
       </c>
     </row>
@@ -1302,39 +1302,39 @@
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr">
         <is>
-          <t>- Chapter 2 theoretical framework — specifically the productive/unproductive labor classification applied to NIPA — must remain operational for the ratio to be interpretable; any drift in the S503 upstream build will propagate here</t>
+          <t>- Reference values dict in `series_registry.json` is currently empty (this DPR is the authoritative benchmark record pending registry patch)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
-      <c r="B61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>- Chapter 2 theoretical framework — specifically the productive/unproductive labor classification applied to NIPA — must remain operational for the ratio to be interpretable; any drift in the S503 upstream build will propagate here</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>## Cross-references</t>
-        </is>
-      </c>
+      <c r="B62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
-      <c r="B63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>## Cross-references</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>- Upstream dependencies: S503 (Marxian GFP*), S501 (Total Product TP*), S502 (Intermediate inputs)</t>
-        </is>
-      </c>
+      <c r="B64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
-          <t>- Downstream consumers: S901 (Chapter-9-style summary table)</t>
+          <t>- Upstream dependencies: S503 (Marxian GFP*), S501 (Total Product TP*), S502 (Intermediate inputs)</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
-          <t>- Related external studies: Eisner (1988) extended accounts; Nordhaus-Tobin (1972) MEW; Jorgenson-Fraumeni human-capital accounts; Kendrick (1976); Ruggles-Ruggles (1970); Zolotas (1981)</t>
+          <t>- Downstream consumers: S901 (Chapter-9-style summary table)</t>
         </is>
       </c>
     </row>
@@ -1350,45 +1350,53 @@
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
-          <t>- Conceptually adjacent series: ES1101 / ES1102 (ST 1987 net-social-wage decomposition) for the productive/unproductive boundary on the labor side</t>
+          <t>- Related external studies: Eisner (1988) extended accounts; Nordhaus-Tobin (1972) MEW; Jorgenson-Fraumeni human-capital accounts; Kendrick (1976); Ruggles-Ruggles (1970); Zolotas (1981)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
-      <c r="B68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>- Conceptually adjacent series: XS1101 / XS1102 (ST 1987 net-social-wage decomposition) for the productive/unproductive boundary on the labor side</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>## Provenance trail</t>
-        </is>
-      </c>
+      <c r="B69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
-      <c r="B70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>## Provenance trail</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>- **Original research**: `Technical/research/S201_research.json`, researcher `opus_agent`, 2026-05-06; ported from `ST2/research/T201_research.json` on 2026-05-14; verbatim quotes backfilled 2026-05-19 (task `D3_RMWND_quotes_ch7_etc`)</t>
-        </is>
-      </c>
+      <c r="B71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
-          <t>- **DPR enriched**: 2026-05-23 by Stage-3 cohort-1 ingestion agent (cohort agent 4); sources read = research JSON + registry entry + KB chunks 03/04/05/26 cited via the research JSON</t>
+          <t>- **Original research**: `Technical/research/S201_research.json`, researcher `opus_agent`, 2026-05-06; ported from `ST2/research/T201_research.json` on 2026-05-14; verbatim quotes backfilled 2026-05-19 (task `D3_RMWND_quotes_ch7_etc`)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
+        <is>
+          <t>- **DPR enriched**: 2026-05-23 by Stage-3 cohort-1 ingestion agent (cohort agent 4); sources read = research JSON + registry entry + KB chunks 03/04/05/26 cited via the research JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
         <is>
           <t>- **Anu Framework stage**: Stage 3 INGESTION (cohort 1, failing chapters); ingestion gate IDs P31/P32</t>
         </is>
@@ -1405,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -1489,7 +1497,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>It should be emphasized once again that the classical distinction between production and nonproduction labor is essentially analytical. It is founded on the insight that certain types of labor share a common property with the activity of consumption -- namely, that in their performance they use up a portion of existing wealth without directly resulting in the creation of new wealth.</t>
+          <t>It must be emphasized once again that the classical distinction between production and nonproduction labor is essentially analytical. It is founded on the insight that certain types of labor share a common property with the activity of consumption -- namely, that in their performance they use up a portion of existing wealth without directly resulting in the creation of new wealth.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1506,7 +1514,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The location of the dividing line between production and nonproduction activities has other implications as well. It changes the very measures of net product, surplus product, consumption, investment, and productivity. The observed trends of these and many other critical variables are also quite different from those in conventional accounts.</t>
+          <t>The location of the dividing line between production and nonproduction activities has other implications as well. We will find that it changes the very measures of net product, surplus product, consumption, investment, and productivity. The observed trends of these and many other critical variables are also quite different from those in conventional accounts.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1642,12 +1650,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Series registry indicates S201 maps to book Table 2.1 (Alternative GFP Measures), source file ch02/Table2_1_AlternativeGFP.csv, annual data 1948-1989, units in billions of dollars. The series is wave3_planned with deferred reason: 'Wave 3 series — requires Ch2 theoretical framework implementation'. Subseries S201-A represents the digitized book table values.</t>
+          <t>CORRECTION (2026-06-11 reconciliation): S201 is NOT a digitized book table. It is a DERIVED annual ratio series, 1948-1989, computed as GFP_GDP_ratio = S503 (Marxian GFP*) / orthodox GDP, with the numerator from this project's Ch5 build and the denominator from BEA NIPA. It is the project's annual analog of the book's Figure 5.4 ('Ratios of real product measures', p.106) and Table 5.4 row 'GFP*/GNP' (p.100). There is NO book 'Table 2.1' — the book's List of Tables (pp. xi-xiii) has no Table 2.1; Chapter 2 is purely theoretical and contains no tables. The earlier claim that S201 maps to 'book Table 2.1 (Alternative GFP Measures), ch02/Table2_1_AlternativeGFP.csv' was a hallucination and has been removed. The NAME 'Alternative GFP Measures' derives from book Figure 1.1 ('Alternate measures of GFP', p.16), a seven-author cross-section; S201 generalizes that comparison to an annual ratio panel. Units are RATIO (observed 0.773-0.903), not billions of dollars.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>NickyData/series_registry.json, S201 entry</t>
+          <t>S201_DPR.md; ST_1994 Fig 1.1 p.16, Fig 5.4 p.106, Table 5.4 p.100; series_registry.json S201 entry</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1667,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>The S201 series is wave3_planned and has not yet been implemented. Construction requires Step 1: load subseries S201-A (book Table 2.1 digitized values). No extension beyond 1989 is currently specified. The series requires the Ch2 theoretical framework to be operational, meaning the productive/unproductive labor classification applied to national accounts data in Chapter 3 must be implemented first.</t>
+          <t>S201 covers the book period 1948-1989 only because its numerator S503 (Marxian GFP*) is built from the book's IO/NIPA tables, which span 1948-1989. The TRIAGE_PRESCREEN COVERAGE_SHORT/COVERAGE_START flags (expected 1929-2025) are FALSE POSITIVES: there is no 1929-2025 source for a Marxian-GFP/GDP ratio without a post-1989 productive/unproductive concordance, which this series does not implement (extension: null). The 1948-1989 span is the correct and intended coverage.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>NickyData/series_registry.json, S201 entry; ST_1994, Ch2</t>
+          <t>S201_DPR.md; ST_1994, Ch5 Tables E.1/E.2</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1765,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>S201 (Alternative GFP Measures) reproduces Shaikh and Tonak's Figure 1.1 comparison of seven gross final product estimates relative to official BEA GNP for the mid-1960s benchmark. The ST measure applies a classical production/nonproduction distinction: trading, military, police, and administrative activities are excluded as social consumption rather than counted as output, in contrast to orthodox GDP/GNP. The series maps to book Table 2.1 (annual data, 1948-1989, billions of dollars) and is currently wave3_planned, requiring digitization of the book table and implementation of the Chapter 2 theoretical framework — specifically the productive/unproductive labor classification — before construction can proceed. The planned construction consists of a single load step (subseries S201-A from ch02/Table2_1_AlternativeGFP.csv) with no current extension beyond 1989.</t>
+          <t>S201 (Alternative GFP Measures) is the annual ratio of the Shaikh-Tonak Marxian Gross Final Product (GFP*, = this project's S503) to orthodox GDP, 1948-1989. It generalizes the book's Figure 1.1 single-benchmark comparison of seven GFP estimates into an annual time series showing how the Marxian-to-orthodox product ratio evolves: it declines from about 0.903 (1948) to 0.773 (1989), indicating that activities the classical framework treats as social consumption (finance, trade margins, government administration) grow faster than productive output over the postwar period. The classical production/nonproduction distinction is the substantive basis: trading, military, police, and administrative activities are excluded as social consumption rather than counted as output. The numerator S503 is built upstream from the book's Ch5 IO/NIPA tables (E.1/E.2); the denominator is BEA NIPA GDP. Units are a ratio. There is no extension beyond 1989.</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1781,7 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Series is wave3_planned; no source CSV yet exists at ch02/Table2_1_AlternativeGFP.csv</t>
+          <t>S201 is a derived ratio (S503/GDP), not a digitized book table; there is no book 'Table 2.1' (the book has no Table 2.1) and no ch02/Table2_1_AlternativeGFP.csv — the prior 'Table 2.1' provenance was a hallucination, corrected 2026-06-11</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1789,7 @@
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Loader L14 and Processor P15 are specified in registry but not yet implemented</t>
+          <t>Registry top-level units were 'billions_usd' but the data are a RATIO (0.773-0.903) — corrected via triage patch</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1797,7 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Figure 1.1 comparison uses different benchmark years across authors (1965-1969), limiting strict comparability</t>
+          <t>Registry content_type was 'cross_sectional' (conflated with the Figure 1.1 cross-section) but the built series is an annual time_series — corrected via triage patch</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1805,7 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ST preferred pure-market estimate (~121% of GNP) differs from the housework-supplemented estimate (~180%) shown in Figure 1.1 for comparability purposes</t>
+          <t>Figure 1.1 (the namesake) compares seven authors at different benchmark years (1965-1969), limiting strict cross-author comparability; that figure is context, not the S201 data</t>
         </is>
       </c>
     </row>
@@ -1805,31 +1813,31 @@
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
-          <t>No extension methodology specified for post-1989 period</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Reference values and expected range not yet populated in series registry validation block</t>
-        </is>
-      </c>
-    </row>
+          <t>No extension beyond 1989: a post-1989 build would require a NAICS-era productive/unproductive concordance not implemented here (extension: null)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Chapter 2 theoretical framework implementation is a prerequisite for wave 3 work</t>
-        </is>
-      </c>
-    </row>
-    <row r="35"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>cross_references:</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>S501</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>cross_references:</t>
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>S502</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1845,7 @@
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>S501</t>
+          <t>S503</t>
         </is>
       </c>
     </row>
@@ -1845,65 +1853,49 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>S502</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>S503</t>
-        </is>
-      </c>
-    </row>
+          <t>S504</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>S504</t>
-        </is>
-      </c>
-    </row>
-    <row r="41"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>citations:</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ST_1994</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Shaikh, Anwar, and E. Ahmet Tonak. 1994. Measuring the Wealth of Nations. Cambridge University Press.</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>citations:</t>
+          <t>Eisner_1988</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Eisner, Robert. 1988. 'Extended Accounts for National Income and Product.' Journal of Economic Literature 26(4): 1611-1684.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ST_1994</t>
+          <t>Juillard_1988</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
-        <is>
-          <t>Shaikh, Anwar, and E. Ahmet Tonak. 1994. Measuring the Wealth of Nations. Cambridge University Press.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Eisner_1988</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Eisner, Robert. 1988. 'Extended Accounts for National Income and Product.' Journal of Economic Literature 26(4): 1611-1684.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Juillard_1988</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
         <is>
           <t>Juillard, Michel. 1988. Un modèle macro-économique pour l'économie américaine. PhD dissertation. (Input-output database adjustments documented in ST 1994 Appendix A.)</t>
         </is>

</xml_diff>

<commit_message>
Release v2.0: comprehensive review + D-batch book-fidelity decisions
Full series-by-series review (~50 series re-examined and corrected for
provenance, units, content labels, and de-tautologised reference values)
plus the D-batch of book-fidelity construction decisions:

- S514 rebuilt on the book's own r*/u division.
- Chapter-7 K* ships a replication-first primary column + labeled variants.
- S515/S516 employment seam rebuilt (share-primitive candidate (d)).
- NSW family adopts book-faithful Candidate A for 1952-89.
- XS1501-XS1504 rebuilt on Mohun (2014) published shares.

DIVERGENCE_REGISTER grown to 69 entries; anu-doctor 0/0; pytest 93 pass /
2 skip / 2 justified xfail. Adds component-chain + per-value provenance
deliverables (COMPONENT_CHAINS, PROVENANCE_DICTIONARY, I-O concordances).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/extenbooks/S201.xlsx
+++ b/extenbooks/S201.xlsx
@@ -886,11 +886,6 @@
           <t>Book Table</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2.1</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -924,7 +919,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1929-2025</t>
+          <t>1948-1989</t>
         </is>
       </c>
     </row>

</xml_diff>